<commit_message>
doc(bip): update xlsx to match table
</commit_message>
<xml_diff>
--- a/docs/ddust-fee-rates.xlsx
+++ b/docs/ddust-fee-rates.xlsx
@@ -56,31 +56,31 @@
     <t>P2TR</t>
   </si>
   <si>
-    <t>Overhead (b)</t>
+    <t>Overhead (B)</t>
   </si>
   <si>
-    <t>Input (b)</t>
+    <t>Input (B)</t>
   </si>
   <si>
-    <t>OP_RETURN (b)</t>
+    <t>OP_RETURN (B)</t>
   </si>
   <si>
-    <t>Base size (b)</t>
+    <t>Base size (B)</t>
   </si>
   <si>
-    <t>Witness data (b)</t>
+    <t>Witness data (B)</t>
   </si>
   <si>
-    <t>Size (b)</t>
+    <t>Size (B)</t>
   </si>
   <si>
     <t>Weight</t>
   </si>
   <si>
-    <t>Virtual Size (vb)</t>
+    <t>Virtual Size (vB)</t>
   </si>
   <si>
-    <t>Fee rates (sats/vb)</t>
+    <t>Fee rates (sats/vB)</t>
   </si>
 </sst>
 </file>
@@ -1334,10 +1334,10 @@
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D4" s="8">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E4" s="8">
         <v>41</v>
@@ -1377,11 +1377,11 @@
       <c r="B6" s="8"/>
       <c r="C6" s="8" cm="1">
         <f t="array" ref="C6">SUM(C3:C5)</f>
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D6" s="8" cm="1">
         <f t="array" ref="D6">SUM(D3:D5)</f>
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E6" s="8" cm="1">
         <f t="array" ref="E6">SUM(E3:E5)</f>
@@ -1408,10 +1408,10 @@
         <v>0</v>
       </c>
       <c r="E7" s="8">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F7" s="8">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="G7" s="8">
         <v>67</v>
@@ -1424,19 +1424,19 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8" cm="1">
         <f t="array" ref="C8">SUM(C6:C7)</f>
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D8" s="8" cm="1">
         <f t="array" ref="D8">SUM(D6:D7)</f>
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E8" s="8" cm="1">
         <f t="array" ref="E8">SUM(E6:E7)</f>
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F8" s="8" cm="1">
         <f t="array" ref="F8">SUM(F6:F7)</f>
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="G8" s="8" cm="1">
         <f t="array" ref="G8">SUM(G6:G7)</f>
@@ -1450,19 +1450,19 @@
       <c r="B9" s="8"/>
       <c r="C9" s="8" cm="1">
         <f t="array" ref="C9">C6*4</f>
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="D9" s="8" cm="1">
         <f t="array" ref="D9">D6*4</f>
-        <v>1264</v>
+        <v>1256</v>
       </c>
       <c r="E9" s="8" cm="1">
         <f t="array" ref="E9">(E6*4)+E7+2</f>
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F9" s="8" cm="1">
         <f t="array" ref="F9">(F6*4)+F7+2</f>
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="G9" s="8" cm="1">
         <f t="array" ref="G9">(G6*4)+G7+2</f>
@@ -1476,19 +1476,19 @@
       <c r="B10" s="8"/>
       <c r="C10" s="8" cm="1">
         <f t="array" ref="C10">C9/4</f>
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D10" s="8" cm="1">
         <f t="array" ref="D10">D9/4</f>
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E10" s="8" cm="1">
         <f t="array" ref="E10">E9/4</f>
-        <v>92.5</v>
+        <v>92.25</v>
       </c>
       <c r="F10" s="8" cm="1">
         <f t="array" ref="F10">F9/4</f>
-        <v>129.25</v>
+        <v>128.5</v>
       </c>
       <c r="G10" s="8" cm="1">
         <f t="array" ref="G10">G9/4</f>
@@ -1522,19 +1522,19 @@
       </c>
       <c r="C13" s="8" cm="1">
         <f t="array" ref="C13">$B13/ROUND(C$10,2)</f>
-        <v>1.7396449704142</v>
+        <v>1.75</v>
       </c>
       <c r="D13" s="8" cm="1">
         <f t="array" ref="D13">$B13/ROUND(D$10,2)</f>
-        <v>0.930379746835443</v>
+        <v>0.936305732484076</v>
       </c>
       <c r="E13" s="8" cm="1">
         <f t="array" ref="E13">$B13/ROUND(E$10,2)</f>
-        <v>3.17837837837838</v>
+        <v>3.1869918699187</v>
       </c>
       <c r="F13" s="8" cm="1">
         <f t="array" ref="F13">$B13/ROUND(F$10,2)</f>
-        <v>2.27466150870406</v>
+        <v>2.28793774319066</v>
       </c>
       <c r="G13" s="8" cm="1">
         <f t="array" ref="G13">$B13/ROUND(G$10,2)</f>
@@ -1548,19 +1548,19 @@
       </c>
       <c r="C14" s="8" cm="1">
         <f t="array" ref="C14">$B14/ROUND(C$10,2)</f>
-        <v>1.77514792899408</v>
+        <v>1.78571428571429</v>
       </c>
       <c r="D14" s="8" cm="1">
         <f t="array" ref="D14">$B14/ROUND(D$10,2)</f>
-        <v>0.949367088607595</v>
+        <v>0.955414012738854</v>
       </c>
       <c r="E14" s="8" cm="1">
         <f t="array" ref="E14">$B14/ROUND(E$10,2)</f>
-        <v>3.24324324324324</v>
+        <v>3.2520325203252</v>
       </c>
       <c r="F14" s="8" cm="1">
         <f t="array" ref="F14">$B14/ROUND(F$10,2)</f>
-        <v>2.321083172147</v>
+        <v>2.33463035019455</v>
       </c>
       <c r="G14" s="8" cm="1">
         <f t="array" ref="G14">$B14/ROUND(G$10,2)</f>
@@ -1574,19 +1574,19 @@
       </c>
       <c r="C15" s="8" cm="1">
         <f t="array" ref="C15">$B15/ROUND(C$10,2)</f>
-        <v>1.92307692307692</v>
+        <v>1.93452380952381</v>
       </c>
       <c r="D15" s="8" cm="1">
         <f t="array" ref="D15">$B15/ROUND(D$10,2)</f>
-        <v>1.02848101265823</v>
+        <v>1.03503184713376</v>
       </c>
       <c r="E15" s="8" cm="1">
         <f t="array" ref="E15">$B15/ROUND(E$10,2)</f>
-        <v>3.51351351351351</v>
+        <v>3.5230352303523</v>
       </c>
       <c r="F15" s="8" cm="1">
         <f t="array" ref="F15">$B15/ROUND(F$10,2)</f>
-        <v>2.51450676982592</v>
+        <v>2.52918287937743</v>
       </c>
       <c r="G15" s="8" cm="1">
         <f t="array" ref="G15">$B15/ROUND(G$10,2)</f>
@@ -1600,19 +1600,19 @@
       </c>
       <c r="C16" s="8" cm="1">
         <f t="array" ref="C16">$B16/ROUND(C$10,2)</f>
-        <v>1.95266272189349</v>
+        <v>1.96428571428571</v>
       </c>
       <c r="D16" s="8" cm="1">
         <f t="array" ref="D16">$B16/ROUND(D$10,2)</f>
-        <v>1.04430379746835</v>
+        <v>1.05095541401274</v>
       </c>
       <c r="E16" s="8" cm="1">
         <f t="array" ref="E16">$B16/ROUND(E$10,2)</f>
-        <v>3.56756756756757</v>
+        <v>3.57723577235772</v>
       </c>
       <c r="F16" s="8" cm="1">
         <f t="array" ref="F16">$B16/ROUND(F$10,2)</f>
-        <v>2.5531914893617</v>
+        <v>2.56809338521401</v>
       </c>
       <c r="G16" s="8" cm="1">
         <f t="array" ref="G16">$B16/ROUND(G$10,2)</f>

</xml_diff>

<commit_message>
ref: always use OP_RETURN ash output
</commit_message>
<xml_diff>
--- a/docs/ddust-fee-rates.xlsx
+++ b/docs/ddust-fee-rates.xlsx
@@ -62,7 +62,7 @@
     <t>Input (B)</t>
   </si>
   <si>
-    <t>OP_RETURN (B)</t>
+    <t>OP_RETURN  “ash” (B)</t>
   </si>
   <si>
     <t>Base size (B)</t>
@@ -1271,7 +1271,8 @@
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="7" width="16.3516" style="1" customWidth="1"/>
+    <col min="1" max="1" width="21.2812" style="1" customWidth="1"/>
+    <col min="2" max="7" width="16.3516" style="1" customWidth="1"/>
     <col min="8" max="16384" width="16.3516" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1355,10 +1356,10 @@
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D5" s="8">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E5" s="8">
         <v>14</v>
@@ -1377,11 +1378,11 @@
       <c r="B6" s="8"/>
       <c r="C6" s="8" cm="1">
         <f t="array" ref="C6">SUM(C3:C5)</f>
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D6" s="8" cm="1">
         <f t="array" ref="D6">SUM(D3:D5)</f>
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E6" s="8" cm="1">
         <f t="array" ref="E6">SUM(E3:E5)</f>
@@ -1424,11 +1425,11 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8" cm="1">
         <f t="array" ref="C8">SUM(C6:C7)</f>
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D8" s="8" cm="1">
         <f t="array" ref="D8">SUM(D6:D7)</f>
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E8" s="8" cm="1">
         <f t="array" ref="E8">SUM(E6:E7)</f>
@@ -1450,11 +1451,11 @@
       <c r="B9" s="8"/>
       <c r="C9" s="8" cm="1">
         <f t="array" ref="C9">C6*4</f>
-        <v>672</v>
+        <v>684</v>
       </c>
       <c r="D9" s="8" cm="1">
         <f t="array" ref="D9">D6*4</f>
-        <v>1256</v>
+        <v>1268</v>
       </c>
       <c r="E9" s="8" cm="1">
         <f t="array" ref="E9">(E6*4)+E7+2</f>
@@ -1476,11 +1477,11 @@
       <c r="B10" s="8"/>
       <c r="C10" s="8" cm="1">
         <f t="array" ref="C10">C9/4</f>
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D10" s="8" cm="1">
         <f t="array" ref="D10">D9/4</f>
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E10" s="8" cm="1">
         <f t="array" ref="E10">E9/4</f>
@@ -1522,11 +1523,11 @@
       </c>
       <c r="C13" s="8" cm="1">
         <f t="array" ref="C13">$B13/ROUND(C$10,2)</f>
-        <v>1.75</v>
+        <v>1.71929824561404</v>
       </c>
       <c r="D13" s="8" cm="1">
         <f t="array" ref="D13">$B13/ROUND(D$10,2)</f>
-        <v>0.936305732484076</v>
+        <v>0.927444794952681</v>
       </c>
       <c r="E13" s="8" cm="1">
         <f t="array" ref="E13">$B13/ROUND(E$10,2)</f>
@@ -1548,11 +1549,11 @@
       </c>
       <c r="C14" s="8" cm="1">
         <f t="array" ref="C14">$B14/ROUND(C$10,2)</f>
-        <v>1.78571428571429</v>
+        <v>1.75438596491228</v>
       </c>
       <c r="D14" s="8" cm="1">
         <f t="array" ref="D14">$B14/ROUND(D$10,2)</f>
-        <v>0.955414012738854</v>
+        <v>0.946372239747634</v>
       </c>
       <c r="E14" s="8" cm="1">
         <f t="array" ref="E14">$B14/ROUND(E$10,2)</f>
@@ -1574,11 +1575,11 @@
       </c>
       <c r="C15" s="8" cm="1">
         <f t="array" ref="C15">$B15/ROUND(C$10,2)</f>
-        <v>1.93452380952381</v>
+        <v>1.90058479532164</v>
       </c>
       <c r="D15" s="8" cm="1">
         <f t="array" ref="D15">$B15/ROUND(D$10,2)</f>
-        <v>1.03503184713376</v>
+        <v>1.02523659305994</v>
       </c>
       <c r="E15" s="8" cm="1">
         <f t="array" ref="E15">$B15/ROUND(E$10,2)</f>
@@ -1600,11 +1601,11 @@
       </c>
       <c r="C16" s="8" cm="1">
         <f t="array" ref="C16">$B16/ROUND(C$10,2)</f>
-        <v>1.96428571428571</v>
+        <v>1.92982456140351</v>
       </c>
       <c r="D16" s="8" cm="1">
         <f t="array" ref="D16">$B16/ROUND(D$10,2)</f>
-        <v>1.05095541401274</v>
+        <v>1.0410094637224</v>
       </c>
       <c r="E16" s="8" cm="1">
         <f t="array" ref="E16">$B16/ROUND(E$10,2)</f>

</xml_diff>